<commit_message>
final ubah date dan number
</commit_message>
<xml_diff>
--- a/template_pst.xlsx
+++ b/template_pst.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29929"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2273001F-4F13-479A-B3C5-5C25DB49F753}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CFCD3240-48E7-40F9-9C42-8D6CE38002A7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -11,21 +11,33 @@
     <sheet name="Form Perjalanan Dinas" sheetId="2" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'Form Perjalanan Dinas'!$A$1:$L$56</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'Form Perjalanan Dinas'!$A1:$L56</definedName>
   </definedNames>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="68" uniqueCount="61">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="76" uniqueCount="66">
   <si>
     <t xml:space="preserve">KEMENTERIAN PERTANIAN </t>
   </si>
   <si>
+    <t>Dibuat Oleh :</t>
+  </si>
+  <si>
+    <t>gusti.yasfin@pertanian.go.id</t>
+  </si>
+  <si>
     <t>BADAN PERAKITAN DAN MODERNISASI PERTANIAN</t>
   </si>
   <si>
+    <t>Dibuat Pada :</t>
+  </si>
+  <si>
+    <t>15/04/2026, 08.22.20</t>
+  </si>
+  <si>
     <t>PUSAT PERAKITAN DAN MODERNISASI PERTANIAN PERKEBUNAN</t>
   </si>
   <si>
@@ -59,22 +71,25 @@
     <t>Golongan</t>
   </si>
   <si>
-    <t>Herlina Saragih</t>
-  </si>
-  <si>
-    <t>PENGADMINISTRASI PERKANTORAN</t>
+    <t>Ghozy Nabil Harits, S.P.</t>
+  </si>
+  <si>
+    <t>CALON PENGAWAS BENIH TANAMAN AHLI PERTAMA</t>
   </si>
   <si>
     <t>III/a</t>
   </si>
   <si>
-    <t>Risma Damayanti, A.MD</t>
-  </si>
-  <si>
-    <t>PENGAWAS BENIH TANAMAN TERAMPIL</t>
-  </si>
-  <si>
-    <t>II/c</t>
+    <t>Zahran Muzzaki, S.Tr.Kom.</t>
+  </si>
+  <si>
+    <t>CALON PRANATA HUBUNGAN MASYARAKAT AHLI PERTAMA</t>
+  </si>
+  <si>
+    <t>Dara Fakhira Dwimareta, S.P.</t>
+  </si>
+  <si>
+    <t>CALON PENGAWAS MUTU HASIL PERTANIAN AHLI PERTAMA</t>
   </si>
   <si>
     <t>Sesuai  dengan SURAT TUGAS ,    No.              /ST/SPD/Kp.410/H.4/4/2026</t>
@@ -86,13 +101,13 @@
     <t>:</t>
   </si>
   <si>
-    <t>Jakarta</t>
+    <t xml:space="preserve">Jakarta </t>
   </si>
   <si>
     <t xml:space="preserve">Maksud Perjalanan Dinas                  </t>
   </si>
   <si>
-    <t>Koordinasi</t>
+    <t xml:space="preserve">Koordinasi Dengan Ditjen Perkebunan </t>
   </si>
   <si>
     <r>
@@ -116,6 +131,9 @@
     <t xml:space="preserve">Tanggal Berangkat / Kembali        </t>
   </si>
   <si>
+    <t>16/4/2026</t>
+  </si>
+  <si>
     <t>s/d</t>
   </si>
   <si>
@@ -167,6 +185,9 @@
     <t xml:space="preserve">Rp.  </t>
   </si>
   <si>
+    <t>...……………………</t>
+  </si>
+  <si>
     <t>2.</t>
   </si>
   <si>
@@ -176,9 +197,6 @@
     <t>Rp.</t>
   </si>
   <si>
-    <t>...……………………</t>
-  </si>
-  <si>
     <t>3.</t>
   </si>
   <si>
@@ -209,10 +227,7 @@
     <t>PUMK Perjalanan</t>
   </si>
   <si>
-    <t>Dibuat Oleh :</t>
-  </si>
-  <si>
-    <t>Dibuat Pada :</t>
+    <t>`</t>
   </si>
 </sst>
 </file>
@@ -220,7 +235,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="166" formatCode="[$-421]dd\ mmmm\ yyyy;@"/>
+    <numFmt numFmtId="164" formatCode="[$-421]dd\ mmmm\ yyyy;@"/>
   </numFmts>
   <fonts count="15" x14ac:knownFonts="1">
     <font>
@@ -239,6 +254,12 @@
     <font>
       <sz val="14"/>
       <color indexed="18"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
       <name val="Arial"/>
       <family val="2"/>
     </font>
@@ -310,12 +331,6 @@
       <name val="Arial"/>
       <family val="2"/>
     </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Arial"/>
-      <family val="2"/>
-    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -325,7 +340,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="32">
+  <borders count="34">
     <border>
       <left/>
       <right/>
@@ -708,214 +723,249 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="79">
+  <cellXfs count="84">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="3" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="33" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="14" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="166" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1247,18 +1297,19 @@
     <col min="2" max="2" width="4.81640625" customWidth="1"/>
     <col min="3" max="3" width="25" customWidth="1"/>
     <col min="4" max="4" width="1.81640625" customWidth="1"/>
-    <col min="5" max="5" width="9.453125" customWidth="1"/>
+    <col min="5" max="5" width="8" customWidth="1"/>
     <col min="6" max="6" width="9.26953125" customWidth="1"/>
     <col min="7" max="7" width="3.7265625" customWidth="1"/>
-    <col min="8" max="8" width="25.81640625" style="1" customWidth="1"/>
-    <col min="9" max="9" width="28.54296875" customWidth="1"/>
-    <col min="10" max="10" width="3.6328125" customWidth="1"/>
+    <col min="8" max="8" width="37.7265625" style="1" customWidth="1"/>
+    <col min="9" max="9" width="25.08984375" customWidth="1"/>
+    <col min="10" max="10" width="0.1796875" customWidth="1"/>
     <col min="11" max="11" width="14.6328125" hidden="1" customWidth="1"/>
-    <col min="12" max="13" width="9.1796875" hidden="1" customWidth="1"/>
+    <col min="12" max="12" width="9.1796875" hidden="1" customWidth="1"/>
+    <col min="13" max="13" width="3.26953125" hidden="1" customWidth="1"/>
     <col min="14" max="14" width="13.08984375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" ht="17.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:15" ht="17.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C1" s="40" t="s">
         <v>0</v>
       </c>
@@ -1268,14 +1319,16 @@
       <c r="G1" s="40"/>
       <c r="H1" s="40"/>
       <c r="I1" s="40"/>
-      <c r="N1" s="78" t="s">
-        <v>59</v>
-      </c>
-      <c r="O1" s="78"/>
-    </row>
-    <row r="2" spans="1:15" ht="17.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="N1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="O1" s="2" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2" spans="1:15" ht="17.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C2" s="41" t="s">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D2" s="41"/>
       <c r="E2" s="41"/>
@@ -1283,16 +1336,18 @@
       <c r="G2" s="41"/>
       <c r="H2" s="41"/>
       <c r="I2" s="41"/>
-      <c r="J2" s="2"/>
-      <c r="L2" s="2"/>
-      <c r="N2" s="78" t="s">
-        <v>60</v>
-      </c>
-      <c r="O2" s="78"/>
+      <c r="J2" s="3"/>
+      <c r="L2" s="3"/>
+      <c r="N2" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="O2" s="2" t="s">
+        <v>5</v>
+      </c>
     </row>
     <row r="3" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C3" s="42" t="s">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="D3" s="42"/>
       <c r="E3" s="42"/>
@@ -1300,12 +1355,12 @@
       <c r="G3" s="42"/>
       <c r="H3" s="42"/>
       <c r="I3" s="42"/>
-      <c r="J3" s="3"/>
-      <c r="L3" s="3"/>
+      <c r="J3" s="4"/>
+      <c r="L3" s="4"/>
     </row>
     <row r="4" spans="1:15" x14ac:dyDescent="0.25">
       <c r="C4" s="43" t="s">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="D4" s="43"/>
       <c r="E4" s="43"/>
@@ -1316,7 +1371,7 @@
     </row>
     <row r="5" spans="1:15" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C5" s="44" t="s">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="D5" s="44"/>
       <c r="E5" s="44"/>
@@ -1327,7 +1382,7 @@
     </row>
     <row r="6" spans="1:15" ht="12" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C6" s="44" t="s">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="D6" s="44"/>
       <c r="E6" s="44"/>
@@ -1335,426 +1390,436 @@
       <c r="G6" s="44"/>
       <c r="H6" s="44"/>
       <c r="I6" s="44"/>
-      <c r="J6" s="4"/>
-      <c r="L6" s="4"/>
+      <c r="J6" s="5"/>
+      <c r="L6" s="5"/>
     </row>
     <row r="7" spans="1:15" ht="10" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="5"/>
-      <c r="B7" s="5"/>
-      <c r="C7" s="5"/>
-      <c r="D7" s="5"/>
-      <c r="E7" s="5"/>
-      <c r="F7" s="5"/>
-      <c r="H7" s="5"/>
+      <c r="A7" s="6"/>
+      <c r="B7" s="6"/>
+      <c r="C7" s="6"/>
+      <c r="D7" s="6"/>
+      <c r="E7" s="6"/>
+      <c r="F7" s="6"/>
+      <c r="H7" s="6"/>
     </row>
     <row r="8" spans="1:15" ht="10" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="5"/>
-      <c r="B8" s="5"/>
-      <c r="C8" s="5"/>
-      <c r="D8" s="5"/>
-      <c r="E8" s="5"/>
-      <c r="F8" s="5"/>
-      <c r="H8" s="5"/>
+      <c r="A8" s="6"/>
+      <c r="B8" s="6"/>
+      <c r="C8" s="6"/>
+      <c r="D8" s="6"/>
+      <c r="E8" s="6"/>
+      <c r="F8" s="6"/>
+      <c r="H8" s="6"/>
     </row>
     <row r="9" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A9" s="6"/>
-      <c r="B9" s="7" t="s">
-        <v>6</v>
-      </c>
-      <c r="C9" s="6"/>
-      <c r="D9" s="6"/>
-      <c r="E9" s="6"/>
-      <c r="F9" s="6"/>
-      <c r="G9" s="6"/>
-      <c r="H9" s="6"/>
+      <c r="A9" s="7"/>
+      <c r="B9" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="C9" s="7"/>
+      <c r="D9" s="7"/>
+      <c r="E9" s="7"/>
+      <c r="F9" s="7"/>
+      <c r="G9" s="7"/>
+      <c r="H9" s="7"/>
     </row>
     <row r="10" spans="1:15" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B10" s="6" t="s">
-        <v>7</v>
-      </c>
-      <c r="C10" s="8"/>
-      <c r="D10" s="8"/>
-      <c r="E10" s="8"/>
-      <c r="F10" s="8"/>
-      <c r="G10" s="7"/>
-      <c r="H10" s="7"/>
+      <c r="B10" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="C10" s="9"/>
+      <c r="D10" s="9"/>
+      <c r="E10" s="9"/>
+      <c r="F10" s="9"/>
+      <c r="G10" s="8"/>
+      <c r="H10" s="8"/>
     </row>
     <row r="11" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="B11" s="6"/>
-      <c r="C11" s="6"/>
-      <c r="D11" s="6"/>
-      <c r="E11" s="6"/>
-      <c r="F11" s="6"/>
-      <c r="G11" s="6"/>
-      <c r="H11" s="9"/>
+      <c r="B11" s="7"/>
+      <c r="C11" s="7"/>
+      <c r="D11" s="7"/>
+      <c r="E11" s="7"/>
+      <c r="F11" s="7"/>
+      <c r="G11" s="7"/>
+      <c r="H11" s="10"/>
     </row>
     <row r="12" spans="1:15" x14ac:dyDescent="0.35">
-      <c r="A12" s="10"/>
+      <c r="A12" s="11"/>
       <c r="B12" s="51" t="s">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="C12" s="45" t="s">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="D12" s="46"/>
-      <c r="E12" s="11"/>
+      <c r="E12" s="12"/>
       <c r="F12" s="45" t="s">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="G12" s="46"/>
       <c r="H12" s="47"/>
-      <c r="I12" s="12" t="s">
-        <v>11</v>
+      <c r="I12" s="13" t="s">
+        <v>15</v>
       </c>
     </row>
     <row r="13" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A13" s="10"/>
+      <c r="A13" s="11"/>
       <c r="B13" s="52"/>
       <c r="C13" s="48"/>
       <c r="D13" s="49"/>
-      <c r="E13" s="10"/>
+      <c r="E13" s="11"/>
       <c r="F13" s="48"/>
       <c r="G13" s="49"/>
       <c r="H13" s="50"/>
-      <c r="I13" s="13" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="14" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="14"/>
-      <c r="B14" s="15">
+      <c r="I13" s="14" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="14" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A14" s="15"/>
+      <c r="B14" s="16">
         <v>1</v>
       </c>
       <c r="C14" s="53" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="D14" s="54"/>
       <c r="E14" s="55"/>
       <c r="F14" s="56" t="s">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="G14" s="56"/>
       <c r="H14" s="56"/>
-      <c r="I14" s="16" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="15" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A15" s="14"/>
-      <c r="B15" s="17">
+      <c r="I14" s="17" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="15" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A15" s="15"/>
+      <c r="B15" s="18">
         <v>2</v>
       </c>
       <c r="C15" s="57" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="D15" s="58"/>
       <c r="E15" s="59"/>
       <c r="F15" s="60" t="s">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="G15" s="60"/>
       <c r="H15" s="60"/>
-      <c r="I15" s="19" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="16" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A16" s="14"/>
-      <c r="B16" s="17"/>
-      <c r="C16" s="61"/>
-      <c r="D16" s="62"/>
-      <c r="E16" s="63"/>
-      <c r="F16" s="60"/>
+      <c r="I15" s="20" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="16" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A16" s="15"/>
+      <c r="B16" s="18">
+        <v>3</v>
+      </c>
+      <c r="C16" s="57" t="s">
+        <v>22</v>
+      </c>
+      <c r="D16" s="58"/>
+      <c r="E16" s="59"/>
+      <c r="F16" s="60" t="s">
+        <v>23</v>
+      </c>
       <c r="G16" s="60"/>
       <c r="H16" s="60"/>
-      <c r="I16" s="19"/>
-    </row>
-    <row r="17" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A17" s="10"/>
-      <c r="B17" s="21"/>
-      <c r="C17" s="61"/>
-      <c r="D17" s="62"/>
-      <c r="E17" s="63"/>
+      <c r="I16" s="20" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="17" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A17" s="11"/>
+      <c r="B17" s="22"/>
+      <c r="C17" s="57"/>
+      <c r="D17" s="58"/>
+      <c r="E17" s="59"/>
       <c r="F17" s="60"/>
       <c r="G17" s="60"/>
       <c r="H17" s="60"/>
-      <c r="I17" s="20"/>
-      <c r="J17" s="22"/>
-    </row>
-    <row r="18" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A18" s="10"/>
-      <c r="B18" s="21"/>
-      <c r="C18" s="61"/>
-      <c r="D18" s="62"/>
-      <c r="E18" s="63"/>
+      <c r="I17" s="21"/>
+      <c r="J17" s="23"/>
+    </row>
+    <row r="18" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A18" s="11"/>
+      <c r="B18" s="22" t="s">
+        <v>65</v>
+      </c>
+      <c r="C18" s="57"/>
+      <c r="D18" s="58"/>
+      <c r="E18" s="59"/>
       <c r="F18" s="60"/>
       <c r="G18" s="60"/>
       <c r="H18" s="60"/>
-      <c r="I18" s="20"/>
-      <c r="J18" s="22"/>
-    </row>
-    <row r="19" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A19" s="10"/>
-      <c r="B19" s="21"/>
-      <c r="C19" s="61"/>
-      <c r="D19" s="62"/>
-      <c r="E19" s="63"/>
+      <c r="I18" s="21"/>
+      <c r="J18" s="23"/>
+    </row>
+    <row r="19" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A19" s="11"/>
+      <c r="B19" s="22"/>
+      <c r="C19" s="57"/>
+      <c r="D19" s="58"/>
+      <c r="E19" s="59"/>
       <c r="F19" s="60"/>
       <c r="G19" s="60"/>
       <c r="H19" s="60"/>
-      <c r="I19" s="19"/>
-    </row>
-    <row r="20" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A20" s="10"/>
-      <c r="B20" s="21"/>
-      <c r="C20" s="61"/>
-      <c r="D20" s="62"/>
-      <c r="E20" s="63"/>
+      <c r="I19" s="20"/>
+    </row>
+    <row r="20" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A20" s="11"/>
+      <c r="B20" s="22"/>
+      <c r="C20" s="57"/>
+      <c r="D20" s="58"/>
+      <c r="E20" s="59"/>
       <c r="F20" s="60"/>
       <c r="G20" s="60"/>
       <c r="H20" s="60"/>
-      <c r="I20" s="19"/>
-    </row>
-    <row r="21" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="14"/>
-      <c r="B21" s="23"/>
-      <c r="C21" s="64"/>
-      <c r="D21" s="65"/>
-      <c r="E21" s="66"/>
-      <c r="F21" s="64"/>
-      <c r="G21" s="65"/>
-      <c r="H21" s="66"/>
-      <c r="I21" s="24"/>
-    </row>
-    <row r="22" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="I20" s="20"/>
+    </row>
+    <row r="21" spans="1:10" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A21" s="15"/>
+      <c r="B21" s="24"/>
+      <c r="C21" s="81"/>
+      <c r="D21" s="82"/>
+      <c r="E21" s="83"/>
+      <c r="F21" s="71"/>
+      <c r="G21" s="72"/>
+      <c r="H21" s="73"/>
+      <c r="I21" s="80"/>
+    </row>
+    <row r="22" spans="1:10" ht="15" customHeight="1" thickTop="1" x14ac:dyDescent="0.35">
       <c r="A22" s="25"/>
       <c r="B22" s="26"/>
       <c r="C22" s="27"/>
       <c r="D22" s="27"/>
-      <c r="E22" s="6"/>
-      <c r="F22" s="6"/>
+      <c r="E22" s="7"/>
+      <c r="F22" s="7"/>
       <c r="G22" s="27"/>
       <c r="H22" s="27"/>
       <c r="I22" s="28"/>
     </row>
     <row r="23" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B23" s="29" t="s">
-        <v>19</v>
-      </c>
-      <c r="C23" s="6"/>
-      <c r="D23" s="6"/>
-      <c r="E23" s="6"/>
-      <c r="F23" s="6"/>
-      <c r="G23" s="6"/>
-      <c r="H23" s="6"/>
+        <v>24</v>
+      </c>
+      <c r="C23" s="7"/>
+      <c r="D23" s="7"/>
+      <c r="E23" s="7"/>
+      <c r="F23" s="7"/>
+      <c r="G23" s="7"/>
+      <c r="H23" s="7"/>
     </row>
     <row r="24" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A24" s="6"/>
+      <c r="A24" s="7"/>
       <c r="B24" s="30" t="s">
-        <v>20</v>
-      </c>
-      <c r="C24" s="6"/>
-      <c r="D24" s="6" t="s">
-        <v>21</v>
-      </c>
-      <c r="E24" s="6" t="s">
-        <v>22</v>
-      </c>
-      <c r="F24" s="6"/>
-      <c r="H24" s="6"/>
+        <v>25</v>
+      </c>
+      <c r="C24" s="7"/>
+      <c r="D24" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="E24" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="F24" s="7"/>
+      <c r="H24" s="7"/>
     </row>
     <row r="25" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A25" s="6"/>
+      <c r="A25" s="7"/>
       <c r="B25" s="30" t="s">
-        <v>23</v>
-      </c>
-      <c r="C25" s="6"/>
-      <c r="D25" s="6" t="s">
-        <v>21</v>
-      </c>
-      <c r="E25" s="6" t="s">
-        <v>24</v>
-      </c>
-      <c r="F25" s="6"/>
-      <c r="H25" s="9"/>
+        <v>28</v>
+      </c>
+      <c r="C25" s="7"/>
+      <c r="D25" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="E25" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="F25" s="7"/>
+      <c r="H25" s="10"/>
     </row>
     <row r="26" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="6"/>
-      <c r="B26" s="6"/>
+      <c r="A26" s="7"/>
+      <c r="B26" s="7"/>
       <c r="C26" s="31"/>
-      <c r="D26" s="7"/>
-      <c r="E26" s="6"/>
-      <c r="F26" s="6"/>
-      <c r="G26" s="6"/>
-      <c r="H26" s="6"/>
-    </row>
-    <row r="27" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A27" s="6"/>
+      <c r="D26" s="8"/>
+      <c r="E26" s="7"/>
+      <c r="F26" s="7"/>
+      <c r="G26" s="7"/>
+      <c r="H26" s="7"/>
+    </row>
+    <row r="27" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A27" s="7"/>
       <c r="B27" s="30" t="s">
-        <v>25</v>
-      </c>
-      <c r="C27" s="6"/>
-      <c r="D27" s="6" t="s">
-        <v>21</v>
-      </c>
-      <c r="E27" s="6" t="s">
+        <v>30</v>
+      </c>
+      <c r="C27" s="7"/>
+      <c r="D27" s="7" t="s">
         <v>26</v>
       </c>
-      <c r="H27" s="6"/>
-    </row>
-    <row r="28" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A28" s="6"/>
+      <c r="E27" s="7" t="s">
+        <v>31</v>
+      </c>
+      <c r="H27" s="7"/>
+    </row>
+    <row r="28" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A28" s="7"/>
       <c r="B28" s="30" t="s">
-        <v>27</v>
-      </c>
-      <c r="C28" s="6"/>
-      <c r="D28" s="6" t="s">
-        <v>21</v>
-      </c>
-      <c r="E28" s="76">
-        <v>46135</v>
-      </c>
-      <c r="F28" s="76"/>
+        <v>32</v>
+      </c>
+      <c r="C28" s="7"/>
+      <c r="D28" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="E28" s="63" t="s">
+        <v>33</v>
+      </c>
+      <c r="F28" s="63"/>
       <c r="G28" s="30" t="s">
-        <v>28</v>
-      </c>
-      <c r="H28" s="76">
-        <v>46136</v>
-      </c>
-      <c r="I28" s="76"/>
-    </row>
-    <row r="29" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A29" s="6"/>
+        <v>34</v>
+      </c>
+      <c r="H28" s="63" t="s">
+        <v>33</v>
+      </c>
+      <c r="I28" s="63"/>
+    </row>
+    <row r="29" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A29" s="7"/>
       <c r="B29" s="30" t="s">
-        <v>29</v>
-      </c>
-      <c r="C29" s="6"/>
-      <c r="D29" s="6" t="s">
-        <v>21</v>
-      </c>
-      <c r="E29" s="67"/>
-      <c r="F29" s="67"/>
-      <c r="G29" s="6"/>
-      <c r="H29" s="6"/>
-    </row>
-    <row r="30" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A30" s="6"/>
-      <c r="B30" s="6"/>
+        <v>35</v>
+      </c>
+      <c r="C29" s="7"/>
+      <c r="D29" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="E29" s="64"/>
+      <c r="F29" s="64"/>
+      <c r="G29" s="7"/>
+      <c r="H29" s="7"/>
+    </row>
+    <row r="30" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A30" s="7"/>
+      <c r="B30" s="7"/>
       <c r="C30" s="31"/>
       <c r="D30" s="31"/>
       <c r="E30" s="31"/>
-      <c r="F30" s="6"/>
-      <c r="G30" s="6"/>
-      <c r="H30" s="6"/>
-    </row>
-    <row r="31" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A31" s="6"/>
-      <c r="B31" s="6"/>
-      <c r="C31" s="6"/>
-      <c r="D31" s="6"/>
-      <c r="E31" s="6"/>
-      <c r="F31" s="6"/>
-      <c r="G31" s="6"/>
-      <c r="H31" s="6" t="s">
-        <v>30</v>
+      <c r="F30" s="7"/>
+      <c r="G30" s="7"/>
+      <c r="H30" s="7"/>
+    </row>
+    <row r="31" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A31" s="7"/>
+      <c r="B31" s="7"/>
+      <c r="C31" s="7"/>
+      <c r="D31" s="7"/>
+      <c r="E31" s="7"/>
+      <c r="F31" s="7"/>
+      <c r="G31" s="7"/>
+      <c r="H31" s="7" t="s">
+        <v>36</v>
       </c>
     </row>
     <row r="32" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A32" s="6"/>
-      <c r="B32" s="6" t="s">
-        <v>31</v>
-      </c>
-      <c r="C32" s="6"/>
-      <c r="D32" s="6"/>
-      <c r="E32" s="6"/>
-      <c r="F32" s="6"/>
-      <c r="G32" s="6"/>
-      <c r="H32" s="6" t="s">
-        <v>32</v>
+      <c r="A32" s="7"/>
+      <c r="B32" s="7" t="s">
+        <v>37</v>
+      </c>
+      <c r="C32" s="7"/>
+      <c r="D32" s="7"/>
+      <c r="E32" s="7"/>
+      <c r="F32" s="7"/>
+      <c r="G32" s="7"/>
+      <c r="H32" s="7" t="s">
+        <v>38</v>
       </c>
     </row>
     <row r="33" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A33" s="6"/>
-      <c r="B33" s="6" t="s">
-        <v>33</v>
-      </c>
-      <c r="C33" s="6"/>
-      <c r="D33" s="6"/>
-      <c r="E33" s="6"/>
-      <c r="F33" s="6"/>
-      <c r="G33" s="6"/>
+      <c r="A33" s="7"/>
+      <c r="B33" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="C33" s="7"/>
+      <c r="D33" s="7"/>
+      <c r="E33" s="7"/>
+      <c r="F33" s="7"/>
+      <c r="G33" s="7"/>
       <c r="H33" s="32" t="s">
-        <v>34</v>
+        <v>40</v>
       </c>
     </row>
     <row r="34" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A34" s="6"/>
-      <c r="B34" s="6"/>
-      <c r="C34" s="6"/>
-      <c r="D34" s="6"/>
-      <c r="E34" s="6"/>
-      <c r="F34" s="6"/>
-      <c r="G34" s="6"/>
+      <c r="A34" s="7"/>
+      <c r="B34" s="7"/>
+      <c r="C34" s="7"/>
+      <c r="D34" s="7"/>
+      <c r="E34" s="7"/>
+      <c r="F34" s="7"/>
+      <c r="G34" s="7"/>
       <c r="H34" s="32"/>
     </row>
     <row r="35" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A35" s="6"/>
-      <c r="B35" s="6"/>
-      <c r="C35" s="6"/>
-      <c r="D35" s="6"/>
-      <c r="E35" s="6"/>
-      <c r="F35" s="6"/>
-      <c r="G35" s="6"/>
+      <c r="A35" s="7"/>
+      <c r="B35" s="7"/>
+      <c r="C35" s="7"/>
+      <c r="D35" s="7"/>
+      <c r="E35" s="7"/>
+      <c r="F35" s="7"/>
+      <c r="G35" s="7"/>
       <c r="H35" s="32"/>
       <c r="J35" s="33"/>
     </row>
     <row r="36" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A36" s="6"/>
-      <c r="B36" s="6"/>
-      <c r="C36" s="6"/>
-      <c r="D36" s="6"/>
-      <c r="E36" s="6"/>
-      <c r="F36" s="6"/>
-      <c r="G36" s="6"/>
+      <c r="A36" s="7"/>
+      <c r="B36" s="7"/>
+      <c r="C36" s="7"/>
+      <c r="D36" s="7"/>
+      <c r="E36" s="7"/>
+      <c r="F36" s="7"/>
+      <c r="G36" s="7"/>
       <c r="H36" s="32"/>
       <c r="J36" s="32"/>
     </row>
     <row r="37" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A37" s="6"/>
+      <c r="A37" s="7"/>
       <c r="B37" s="31" t="s">
-        <v>35</v>
-      </c>
-      <c r="C37" s="6"/>
-      <c r="D37" s="6"/>
-      <c r="E37" s="6"/>
+        <v>41</v>
+      </c>
+      <c r="C37" s="7"/>
+      <c r="D37" s="7"/>
+      <c r="E37" s="7"/>
       <c r="F37" s="31"/>
       <c r="G37" s="31"/>
       <c r="H37" s="34" t="s">
-        <v>36</v>
+        <v>42</v>
       </c>
       <c r="J37" s="33"/>
     </row>
     <row r="38" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A38" s="6"/>
+      <c r="A38" s="7"/>
       <c r="B38" s="32" t="s">
-        <v>37</v>
-      </c>
-      <c r="C38" s="6"/>
-      <c r="D38" s="6"/>
-      <c r="E38" s="6"/>
+        <v>43</v>
+      </c>
+      <c r="C38" s="7"/>
+      <c r="D38" s="7"/>
+      <c r="E38" s="7"/>
       <c r="F38" s="32"/>
       <c r="G38" s="32"/>
       <c r="H38" s="32" t="s">
-        <v>38</v>
+        <v>44</v>
       </c>
       <c r="J38" s="32"/>
     </row>
     <row r="39" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A39" s="6"/>
+      <c r="A39" s="7"/>
       <c r="B39" s="32"/>
-      <c r="C39" s="6"/>
-      <c r="D39" s="6"/>
-      <c r="E39" s="6"/>
+      <c r="C39" s="7"/>
+      <c r="D39" s="7"/>
+      <c r="E39" s="7"/>
       <c r="F39" s="32"/>
       <c r="G39" s="32"/>
       <c r="H39" s="32"/>
@@ -1762,226 +1827,228 @@
     </row>
     <row r="40" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A40" s="31" t="s">
-        <v>39</v>
-      </c>
-      <c r="B40" s="6"/>
-      <c r="C40" s="6"/>
-      <c r="D40" s="6"/>
-      <c r="E40" s="6"/>
-      <c r="F40" s="6"/>
-      <c r="G40" s="6"/>
-      <c r="H40" s="6"/>
+        <v>45</v>
+      </c>
+      <c r="B40" s="7"/>
+      <c r="C40" s="7"/>
+      <c r="D40" s="7"/>
+      <c r="E40" s="7"/>
+      <c r="F40" s="7"/>
+      <c r="G40" s="7"/>
+      <c r="H40" s="7"/>
     </row>
     <row r="41" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A41" s="31" t="s">
-        <v>40</v>
-      </c>
-      <c r="B41" s="6"/>
-      <c r="C41" s="6"/>
-      <c r="D41" s="6"/>
-      <c r="E41" s="6"/>
+        <v>46</v>
+      </c>
+      <c r="B41" s="7"/>
+      <c r="C41" s="7"/>
+      <c r="D41" s="7"/>
+      <c r="E41" s="7"/>
       <c r="F41" s="35" t="s">
-        <v>41</v>
-      </c>
-      <c r="G41" s="6"/>
-      <c r="H41" s="6"/>
+        <v>47</v>
+      </c>
+      <c r="G41" s="7"/>
+      <c r="H41" s="7"/>
     </row>
     <row r="42" spans="1:10" ht="22" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A42" s="6"/>
-      <c r="B42" s="6"/>
-      <c r="C42" s="6"/>
-      <c r="D42" s="6"/>
-      <c r="E42" s="6"/>
-      <c r="F42" s="6"/>
-      <c r="G42" s="6"/>
-      <c r="H42" s="6"/>
+      <c r="A42" s="7"/>
+      <c r="B42" s="7"/>
+      <c r="C42" s="7"/>
+      <c r="D42" s="7"/>
+      <c r="E42" s="7"/>
+      <c r="F42" s="7"/>
+      <c r="G42" s="7"/>
+      <c r="H42" s="7"/>
     </row>
     <row r="43" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A43" s="10" t="s">
-        <v>42</v>
-      </c>
-      <c r="B43" s="6" t="s">
-        <v>43</v>
-      </c>
-      <c r="C43" s="6"/>
-      <c r="E43" s="6" t="s">
-        <v>44</v>
-      </c>
-      <c r="F43" s="6" t="s">
+      <c r="A43" s="11" t="s">
         <v>48</v>
       </c>
-      <c r="G43" s="6"/>
-      <c r="H43" s="77"/>
+      <c r="B43" s="7" t="s">
+        <v>49</v>
+      </c>
+      <c r="C43" s="7"/>
+      <c r="E43" s="7" t="s">
+        <v>50</v>
+      </c>
+      <c r="F43" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="G43" s="7"/>
+      <c r="H43" s="36"/>
     </row>
     <row r="44" spans="1:10" ht="22" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A44" s="10"/>
-      <c r="B44" s="6"/>
-      <c r="C44" s="6"/>
-      <c r="E44" s="6"/>
-      <c r="F44" s="6"/>
-      <c r="G44" s="6"/>
-      <c r="H44" s="6"/>
+      <c r="A44" s="11"/>
+      <c r="B44" s="7"/>
+      <c r="C44" s="7"/>
+      <c r="E44" s="7"/>
+      <c r="F44" s="7"/>
+      <c r="G44" s="7"/>
+      <c r="H44" s="7"/>
     </row>
     <row r="45" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A45" s="10" t="s">
-        <v>45</v>
-      </c>
-      <c r="B45" s="6" t="s">
-        <v>46</v>
-      </c>
-      <c r="C45" s="6"/>
-      <c r="E45" s="6" t="s">
-        <v>47</v>
-      </c>
-      <c r="F45" s="77"/>
-      <c r="G45" s="6"/>
-      <c r="H45" s="6"/>
+      <c r="A45" s="11" t="s">
+        <v>52</v>
+      </c>
+      <c r="B45" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="C45" s="7"/>
+      <c r="E45" s="7" t="s">
+        <v>54</v>
+      </c>
+      <c r="F45" s="79">
+        <v>15123</v>
+      </c>
+      <c r="G45" s="7"/>
+      <c r="H45" s="7"/>
     </row>
     <row r="46" spans="1:10" ht="22" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A46" s="10"/>
-      <c r="B46" s="6"/>
-      <c r="C46" s="6"/>
-      <c r="D46" s="6"/>
-      <c r="E46" s="6"/>
-      <c r="F46" s="6"/>
-      <c r="G46" s="6"/>
-      <c r="H46" s="6"/>
+      <c r="A46" s="11"/>
+      <c r="B46" s="7"/>
+      <c r="C46" s="7"/>
+      <c r="D46" s="7"/>
+      <c r="E46" s="7"/>
+      <c r="F46" s="7"/>
+      <c r="G46" s="7"/>
+      <c r="H46" s="7"/>
     </row>
     <row r="47" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A47" s="10" t="s">
-        <v>49</v>
-      </c>
-      <c r="B47" s="6" t="s">
-        <v>50</v>
+      <c r="A47" s="11" t="s">
+        <v>55</v>
+      </c>
+      <c r="B47" s="7" t="s">
+        <v>56</v>
       </c>
       <c r="C47" s="31"/>
       <c r="D47" s="31"/>
-      <c r="E47" s="6" t="s">
+      <c r="E47" s="7" t="s">
+        <v>57</v>
+      </c>
+      <c r="F47" s="7" t="s">
         <v>51</v>
       </c>
-      <c r="F47" s="6" t="s">
-        <v>48</v>
-      </c>
-      <c r="G47" s="6"/>
-      <c r="H47" s="6"/>
+      <c r="G47" s="7"/>
+      <c r="H47" s="7"/>
     </row>
     <row r="48" spans="1:10" ht="22" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A48" s="10"/>
-      <c r="B48" s="6"/>
-      <c r="C48" s="6"/>
-      <c r="D48" s="6"/>
-      <c r="E48" s="6"/>
-      <c r="F48" s="6"/>
-      <c r="G48" s="6"/>
-      <c r="H48" s="6"/>
+      <c r="A48" s="11"/>
+      <c r="B48" s="7"/>
+      <c r="C48" s="7"/>
+      <c r="D48" s="7"/>
+      <c r="E48" s="7"/>
+      <c r="F48" s="7"/>
+      <c r="G48" s="7"/>
+      <c r="H48" s="7"/>
     </row>
     <row r="49" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A49" s="10" t="s">
-        <v>52</v>
-      </c>
-      <c r="B49" s="6" t="s">
-        <v>53</v>
-      </c>
-      <c r="C49" s="6"/>
-      <c r="D49" s="6"/>
-      <c r="E49" s="6" t="s">
+      <c r="A49" s="11" t="s">
+        <v>58</v>
+      </c>
+      <c r="B49" s="7" t="s">
+        <v>59</v>
+      </c>
+      <c r="C49" s="7"/>
+      <c r="D49" s="7"/>
+      <c r="E49" s="7" t="s">
+        <v>57</v>
+      </c>
+      <c r="F49" s="7" t="s">
         <v>51</v>
       </c>
-      <c r="F49" s="6" t="s">
-        <v>48</v>
-      </c>
-      <c r="G49" s="6"/>
-      <c r="H49" s="6"/>
+      <c r="G49" s="7"/>
+      <c r="H49" s="7"/>
     </row>
     <row r="50" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A50" s="6"/>
-      <c r="B50" s="6"/>
-      <c r="C50" s="6"/>
-      <c r="D50" s="6"/>
-      <c r="E50" s="6"/>
-      <c r="F50" s="6"/>
-      <c r="G50" s="6"/>
-      <c r="H50" s="6"/>
+      <c r="A50" s="7"/>
+      <c r="B50" s="7"/>
+      <c r="C50" s="7"/>
+      <c r="D50" s="7"/>
+      <c r="E50" s="7"/>
+      <c r="F50" s="7"/>
+      <c r="G50" s="7"/>
+      <c r="H50" s="7"/>
     </row>
     <row r="51" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A51" s="6"/>
-      <c r="B51" s="6"/>
-      <c r="C51" s="6"/>
-      <c r="D51" s="6"/>
-      <c r="E51" s="6"/>
-      <c r="F51" s="6"/>
-      <c r="G51" s="6"/>
-      <c r="H51" s="6"/>
+      <c r="A51" s="7"/>
+      <c r="B51" s="7"/>
+      <c r="C51" s="7"/>
+      <c r="D51" s="7"/>
+      <c r="E51" s="7"/>
+      <c r="F51" s="7"/>
+      <c r="G51" s="7"/>
+      <c r="H51" s="7"/>
     </row>
     <row r="52" spans="1:9" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A52" s="6"/>
-      <c r="B52" s="68" t="s">
-        <v>54</v>
-      </c>
-      <c r="C52" s="69"/>
-      <c r="D52" s="72" t="s">
-        <v>55</v>
-      </c>
-      <c r="E52" s="73"/>
-      <c r="F52" s="8"/>
-      <c r="G52" s="6"/>
-      <c r="H52" s="6"/>
+      <c r="A52" s="7"/>
+      <c r="B52" s="65" t="s">
+        <v>60</v>
+      </c>
+      <c r="C52" s="66"/>
+      <c r="D52" s="69" t="s">
+        <v>61</v>
+      </c>
+      <c r="E52" s="76"/>
+      <c r="F52" s="70"/>
+      <c r="G52" s="7"/>
+      <c r="H52" s="7"/>
     </row>
     <row r="53" spans="1:9" ht="12" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A53" s="6"/>
-      <c r="B53" s="70"/>
-      <c r="C53" s="71"/>
+      <c r="A53" s="7"/>
+      <c r="B53" s="67"/>
+      <c r="C53" s="68"/>
       <c r="D53" s="74"/>
-      <c r="E53" s="75"/>
-      <c r="F53" s="8"/>
-      <c r="G53" s="6"/>
-      <c r="H53" s="6"/>
+      <c r="E53" s="78"/>
+      <c r="F53" s="75"/>
+      <c r="G53" s="7"/>
+      <c r="H53" s="7"/>
     </row>
     <row r="54" spans="1:9" ht="28.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A54" s="6"/>
-      <c r="B54" s="18" t="s">
-        <v>56</v>
-      </c>
-      <c r="C54" s="36"/>
-      <c r="D54" s="37"/>
-      <c r="E54" s="38"/>
-      <c r="F54" s="6"/>
-      <c r="G54" s="6"/>
-      <c r="H54" s="6"/>
+      <c r="A54" s="7"/>
+      <c r="B54" s="19" t="s">
+        <v>62</v>
+      </c>
+      <c r="C54" s="37"/>
+      <c r="D54" s="77"/>
+      <c r="E54" s="61"/>
+      <c r="F54" s="62"/>
+      <c r="G54" s="7"/>
+      <c r="H54" s="7"/>
     </row>
     <row r="55" spans="1:9" ht="28.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A55" s="6"/>
-      <c r="B55" s="18" t="s">
-        <v>57</v>
-      </c>
-      <c r="C55" s="36"/>
-      <c r="D55" s="37"/>
-      <c r="E55" s="38"/>
-      <c r="F55" s="6"/>
-      <c r="G55" s="6"/>
-      <c r="H55" s="6"/>
+      <c r="A55" s="7"/>
+      <c r="B55" s="19" t="s">
+        <v>63</v>
+      </c>
+      <c r="C55" s="37"/>
+      <c r="D55" s="38"/>
+      <c r="E55" s="61"/>
+      <c r="F55" s="62"/>
+      <c r="G55" s="7"/>
+      <c r="H55" s="7"/>
     </row>
     <row r="56" spans="1:9" ht="28.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A56" s="6"/>
-      <c r="B56" s="18" t="s">
-        <v>58</v>
-      </c>
-      <c r="C56" s="36"/>
-      <c r="D56" s="37"/>
-      <c r="E56" s="38"/>
-      <c r="F56" s="6"/>
-      <c r="G56" s="6"/>
-      <c r="H56" s="6"/>
+      <c r="A56" s="7"/>
+      <c r="B56" s="19" t="s">
+        <v>64</v>
+      </c>
+      <c r="C56" s="37"/>
+      <c r="D56" s="38"/>
+      <c r="E56" s="61"/>
+      <c r="F56" s="62"/>
+      <c r="G56" s="7"/>
+      <c r="H56" s="7"/>
     </row>
     <row r="57" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A57" s="6"/>
-      <c r="B57" s="6"/>
-      <c r="C57" s="6"/>
-      <c r="D57" s="6"/>
-      <c r="E57" s="6"/>
-      <c r="F57" s="6"/>
-      <c r="G57" s="6"/>
-      <c r="H57" s="6"/>
+      <c r="A57" s="7"/>
+      <c r="B57" s="7"/>
+      <c r="C57" s="7"/>
+      <c r="D57" s="7"/>
+      <c r="E57" s="7"/>
+      <c r="F57" s="7"/>
+      <c r="G57" s="7"/>
+      <c r="H57" s="7"/>
     </row>
     <row r="58" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A58" s="39"/>
@@ -1992,203 +2059,206 @@
       <c r="F58" s="39"/>
       <c r="G58" s="39"/>
       <c r="H58" s="39"/>
-      <c r="I58" s="5"/>
+      <c r="I58" s="6"/>
     </row>
     <row r="59" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="H59" s="5"/>
-      <c r="I59" s="5"/>
+      <c r="H59" s="6"/>
+      <c r="I59" s="6"/>
     </row>
     <row r="60" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="H60" s="5"/>
-      <c r="I60" s="5"/>
+      <c r="H60" s="6"/>
+      <c r="I60" s="6"/>
     </row>
     <row r="61" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="H61" s="5"/>
-      <c r="I61" s="5"/>
+      <c r="H61" s="6"/>
+      <c r="I61" s="6"/>
     </row>
     <row r="62" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="H62" s="5"/>
-      <c r="I62" s="5"/>
+      <c r="H62" s="6"/>
+      <c r="I62" s="6"/>
     </row>
     <row r="63" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="H63" s="5"/>
-      <c r="I63" s="5"/>
+      <c r="H63" s="6"/>
+      <c r="I63" s="6"/>
     </row>
     <row r="64" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="H64" s="5"/>
-      <c r="I64" s="5"/>
+      <c r="H64" s="6"/>
+      <c r="I64" s="6"/>
     </row>
     <row r="65" spans="8:9" x14ac:dyDescent="0.35">
-      <c r="H65" s="5"/>
-      <c r="I65" s="5"/>
+      <c r="H65" s="6"/>
+      <c r="I65" s="6"/>
     </row>
     <row r="66" spans="8:9" x14ac:dyDescent="0.35">
-      <c r="H66" s="5"/>
-      <c r="I66" s="5"/>
+      <c r="H66" s="6"/>
+      <c r="I66" s="6"/>
     </row>
     <row r="67" spans="8:9" x14ac:dyDescent="0.35">
-      <c r="H67" s="5"/>
-      <c r="I67" s="5"/>
+      <c r="H67" s="6"/>
+      <c r="I67" s="6"/>
     </row>
     <row r="68" spans="8:9" x14ac:dyDescent="0.35">
-      <c r="H68" s="5"/>
-      <c r="I68" s="5"/>
+      <c r="H68" s="6"/>
+      <c r="I68" s="6"/>
     </row>
     <row r="69" spans="8:9" x14ac:dyDescent="0.35">
-      <c r="H69" s="5"/>
-      <c r="I69" s="5"/>
+      <c r="H69" s="6"/>
+      <c r="I69" s="6"/>
     </row>
     <row r="70" spans="8:9" x14ac:dyDescent="0.35">
-      <c r="H70" s="5"/>
-      <c r="I70" s="5"/>
+      <c r="H70" s="6"/>
+      <c r="I70" s="6"/>
     </row>
     <row r="71" spans="8:9" x14ac:dyDescent="0.35">
-      <c r="H71" s="5"/>
-      <c r="I71" s="5"/>
+      <c r="H71" s="6"/>
+      <c r="I71" s="6"/>
     </row>
     <row r="72" spans="8:9" x14ac:dyDescent="0.35">
-      <c r="H72" s="5"/>
-      <c r="I72" s="5"/>
+      <c r="H72" s="6"/>
+      <c r="I72" s="6"/>
     </row>
     <row r="73" spans="8:9" x14ac:dyDescent="0.35">
-      <c r="H73" s="5"/>
-      <c r="I73" s="5"/>
+      <c r="H73" s="6"/>
+      <c r="I73" s="6"/>
     </row>
     <row r="74" spans="8:9" x14ac:dyDescent="0.35">
-      <c r="H74" s="5"/>
-      <c r="I74" s="5"/>
+      <c r="H74" s="6"/>
+      <c r="I74" s="6"/>
     </row>
     <row r="75" spans="8:9" x14ac:dyDescent="0.35">
-      <c r="H75" s="5"/>
-      <c r="I75" s="5"/>
+      <c r="H75" s="6"/>
+      <c r="I75" s="6"/>
     </row>
     <row r="76" spans="8:9" x14ac:dyDescent="0.35">
-      <c r="H76" s="5"/>
-      <c r="I76" s="5"/>
+      <c r="H76" s="6"/>
+      <c r="I76" s="6"/>
     </row>
     <row r="77" spans="8:9" x14ac:dyDescent="0.35">
-      <c r="H77" s="5"/>
-      <c r="I77" s="5"/>
+      <c r="H77" s="6"/>
+      <c r="I77" s="6"/>
     </row>
     <row r="78" spans="8:9" x14ac:dyDescent="0.35">
-      <c r="H78" s="5"/>
-      <c r="I78" s="5"/>
+      <c r="H78" s="6"/>
+      <c r="I78" s="6"/>
     </row>
     <row r="79" spans="8:9" x14ac:dyDescent="0.35">
-      <c r="H79" s="5"/>
-      <c r="I79" s="5"/>
+      <c r="H79" s="6"/>
+      <c r="I79" s="6"/>
     </row>
     <row r="80" spans="8:9" x14ac:dyDescent="0.35">
-      <c r="H80" s="5"/>
-      <c r="I80" s="5"/>
+      <c r="H80" s="6"/>
+      <c r="I80" s="6"/>
     </row>
     <row r="81" spans="8:9" x14ac:dyDescent="0.35">
-      <c r="H81" s="5"/>
-      <c r="I81" s="5"/>
+      <c r="H81" s="6"/>
+      <c r="I81" s="6"/>
     </row>
     <row r="82" spans="8:9" x14ac:dyDescent="0.35">
-      <c r="H82" s="5"/>
-      <c r="I82" s="5"/>
+      <c r="H82" s="6"/>
+      <c r="I82" s="6"/>
     </row>
     <row r="83" spans="8:9" x14ac:dyDescent="0.35">
-      <c r="H83" s="5"/>
-      <c r="I83" s="5"/>
+      <c r="H83" s="6"/>
+      <c r="I83" s="6"/>
     </row>
     <row r="84" spans="8:9" x14ac:dyDescent="0.35">
-      <c r="H84" s="5"/>
-      <c r="I84" s="5"/>
+      <c r="H84" s="6"/>
+      <c r="I84" s="6"/>
     </row>
     <row r="85" spans="8:9" x14ac:dyDescent="0.35">
-      <c r="H85" s="5"/>
-      <c r="I85" s="5"/>
+      <c r="H85" s="6"/>
+      <c r="I85" s="6"/>
     </row>
     <row r="86" spans="8:9" x14ac:dyDescent="0.35">
-      <c r="H86" s="5"/>
-      <c r="I86" s="5"/>
+      <c r="H86" s="6"/>
+      <c r="I86" s="6"/>
     </row>
     <row r="87" spans="8:9" x14ac:dyDescent="0.35">
-      <c r="H87" s="5"/>
-      <c r="I87" s="5"/>
+      <c r="H87" s="6"/>
+      <c r="I87" s="6"/>
     </row>
     <row r="88" spans="8:9" x14ac:dyDescent="0.35">
-      <c r="H88" s="5"/>
-      <c r="I88" s="5"/>
+      <c r="H88" s="6"/>
+      <c r="I88" s="6"/>
     </row>
     <row r="89" spans="8:9" x14ac:dyDescent="0.35">
-      <c r="H89" s="5"/>
-      <c r="I89" s="5"/>
+      <c r="H89" s="6"/>
+      <c r="I89" s="6"/>
     </row>
     <row r="90" spans="8:9" x14ac:dyDescent="0.35">
-      <c r="H90" s="5"/>
-      <c r="I90" s="5"/>
+      <c r="H90" s="6"/>
+      <c r="I90" s="6"/>
     </row>
     <row r="91" spans="8:9" x14ac:dyDescent="0.35">
-      <c r="H91" s="5"/>
-      <c r="I91" s="5"/>
+      <c r="H91" s="6"/>
+      <c r="I91" s="6"/>
     </row>
     <row r="92" spans="8:9" x14ac:dyDescent="0.35">
-      <c r="H92" s="5"/>
-      <c r="I92" s="5"/>
+      <c r="H92" s="6"/>
+      <c r="I92" s="6"/>
     </row>
     <row r="93" spans="8:9" x14ac:dyDescent="0.35">
-      <c r="H93" s="5"/>
-      <c r="I93" s="5"/>
+      <c r="H93" s="6"/>
+      <c r="I93" s="6"/>
     </row>
     <row r="94" spans="8:9" x14ac:dyDescent="0.35">
-      <c r="H94" s="5"/>
-      <c r="I94" s="5"/>
+      <c r="H94" s="6"/>
+      <c r="I94" s="6"/>
     </row>
     <row r="95" spans="8:9" x14ac:dyDescent="0.35">
-      <c r="H95" s="5"/>
-      <c r="I95" s="5"/>
+      <c r="H95" s="6"/>
+      <c r="I95" s="6"/>
     </row>
     <row r="96" spans="8:9" x14ac:dyDescent="0.35">
-      <c r="H96" s="5"/>
-      <c r="I96" s="5"/>
+      <c r="H96" s="6"/>
+      <c r="I96" s="6"/>
     </row>
     <row r="97" spans="8:9" x14ac:dyDescent="0.35">
-      <c r="H97" s="5"/>
-      <c r="I97" s="5"/>
+      <c r="H97" s="6"/>
+      <c r="I97" s="6"/>
     </row>
     <row r="98" spans="8:9" x14ac:dyDescent="0.35">
-      <c r="H98" s="5"/>
-      <c r="I98" s="5"/>
+      <c r="H98" s="6"/>
+      <c r="I98" s="6"/>
     </row>
     <row r="99" spans="8:9" x14ac:dyDescent="0.35">
-      <c r="H99" s="5"/>
-      <c r="I99" s="5"/>
+      <c r="H99" s="6"/>
+      <c r="I99" s="6"/>
     </row>
     <row r="100" spans="8:9" x14ac:dyDescent="0.35">
-      <c r="H100" s="5"/>
-      <c r="I100" s="5"/>
+      <c r="H100" s="6"/>
+      <c r="I100" s="6"/>
     </row>
     <row r="101" spans="8:9" x14ac:dyDescent="0.35">
-      <c r="H101" s="5"/>
-      <c r="I101" s="5"/>
+      <c r="H101" s="6"/>
+      <c r="I101" s="6"/>
     </row>
     <row r="102" spans="8:9" x14ac:dyDescent="0.35">
-      <c r="H102" s="5"/>
-      <c r="I102" s="5"/>
+      <c r="H102" s="6"/>
+      <c r="I102" s="6"/>
     </row>
     <row r="103" spans="8:9" x14ac:dyDescent="0.35">
-      <c r="H103" s="5"/>
-      <c r="I103" s="5"/>
+      <c r="H103" s="6"/>
+      <c r="I103" s="6"/>
     </row>
     <row r="104" spans="8:9" x14ac:dyDescent="0.35">
-      <c r="H104" s="5"/>
-      <c r="I104" s="5"/>
+      <c r="H104" s="6"/>
+      <c r="I104" s="6"/>
     </row>
   </sheetData>
-  <mergeCells count="31">
+  <mergeCells count="34">
+    <mergeCell ref="E54:F54"/>
+    <mergeCell ref="E55:F55"/>
+    <mergeCell ref="E56:F56"/>
     <mergeCell ref="E29:F29"/>
     <mergeCell ref="B52:C53"/>
-    <mergeCell ref="D52:E53"/>
-    <mergeCell ref="H28:I28"/>
+    <mergeCell ref="D52:F53"/>
     <mergeCell ref="C20:E20"/>
     <mergeCell ref="F20:H20"/>
     <mergeCell ref="C21:E21"/>
     <mergeCell ref="F21:H21"/>
     <mergeCell ref="E28:F28"/>
+    <mergeCell ref="H28:I28"/>
     <mergeCell ref="C17:E17"/>
     <mergeCell ref="F17:H17"/>
     <mergeCell ref="C18:E18"/>

</xml_diff>

<commit_message>
FELINAAA Update template_pst.xlsx v2
</commit_message>
<xml_diff>
--- a/template_pst.xlsx
+++ b/template_pst.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29929"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{135C85B2-F299-4DE6-BE4C-327ECC05E117}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{863C8AC6-0669-4D14-BC13-C64CA93CF6E7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -164,6 +164,12 @@
     <t>NIP. 196904191998031002</t>
   </si>
   <si>
+    <t xml:space="preserve">  CATATAN ANGGARAN</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  JUMLAH ANGGARAN</t>
+  </si>
+  <si>
     <t>TOLAK UKUR  (  6918.EBA.962.051.C.524111 )</t>
   </si>
   <si>
@@ -173,6 +179,9 @@
     <t>Biaya yang telah dipergunakan</t>
   </si>
   <si>
+    <t xml:space="preserve">   Rp  </t>
+  </si>
+  <si>
     <t>...……………………</t>
   </si>
   <si>
@@ -182,6 +191,9 @@
     <t>Biaya yang akan dipergunakan</t>
   </si>
   <si>
+    <t xml:space="preserve">   Rp</t>
+  </si>
+  <si>
     <t>3.</t>
   </si>
   <si>
@@ -207,18 +219,6 @@
   </si>
   <si>
     <t>PUMK Perjalanan</t>
-  </si>
-  <si>
-    <t xml:space="preserve">   Rp</t>
-  </si>
-  <si>
-    <t xml:space="preserve">   Rp  </t>
-  </si>
-  <si>
-    <t xml:space="preserve">  CATATAN ANGGARAN</t>
-  </si>
-  <si>
-    <t xml:space="preserve">  JUMLAH ANGGARAN</t>
   </si>
 </sst>
 </file>
@@ -826,6 +826,9 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
     <xf numFmtId="3" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1"/>
@@ -915,50 +918,47 @@
     <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="14" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="33" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="33" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="3" fontId="14" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1023,49 +1023,61 @@
     </xdr:pic>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
+  <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>0</xdr:col>
-      <xdr:colOff>100263</xdr:colOff>
+      <xdr:colOff>44450</xdr:colOff>
       <xdr:row>6</xdr:row>
-      <xdr:rowOff>57529</xdr:rowOff>
+      <xdr:rowOff>69850</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>9</xdr:col>
-      <xdr:colOff>5452</xdr:colOff>
-      <xdr:row>7</xdr:row>
-      <xdr:rowOff>30280</xdr:rowOff>
+      <xdr:colOff>6350</xdr:colOff>
+      <xdr:row>6</xdr:row>
+      <xdr:rowOff>82550</xdr:rowOff>
     </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="3" name="Picture 2">
+    <xdr:cxnSp macro="">
+      <xdr:nvCxnSpPr>
+        <xdr:cNvPr id="5" name="Straight Connector 4">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{CC8C01F5-93F4-4DD2-9AF7-BF9F629F432D}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{F9304C25-48BC-4D31-CA2C-8F8D7B2C4DD7}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill rotWithShape="1">
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2" cstate="print"/>
-        <a:srcRect t="91492"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
+        <xdr:cNvCxnSpPr/>
+      </xdr:nvCxnSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="100263" y="1243044"/>
-          <a:ext cx="8195618" cy="100841"/>
+          <a:off x="44450" y="1250950"/>
+          <a:ext cx="8248650" cy="12700"/>
         </a:xfrm>
-        <a:prstGeom prst="rect">
+        <a:prstGeom prst="line">
           <a:avLst/>
         </a:prstGeom>
+        <a:ln w="57150" cmpd="thickThin">
+          <a:solidFill>
+            <a:schemeClr val="accent1">
+              <a:lumMod val="75000"/>
+            </a:schemeClr>
+          </a:solidFill>
+        </a:ln>
       </xdr:spPr>
-    </xdr:pic>
+      <xdr:style>
+        <a:lnRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+    </xdr:cxnSp>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
 </xdr:wsDr>
@@ -1349,15 +1361,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:15" ht="17.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C1" s="42" t="s">
+      <c r="C1" s="43" t="s">
         <v>0</v>
       </c>
-      <c r="D1" s="42"/>
-      <c r="E1" s="42"/>
-      <c r="F1" s="42"/>
-      <c r="G1" s="42"/>
-      <c r="H1" s="42"/>
-      <c r="I1" s="42"/>
+      <c r="D1" s="43"/>
+      <c r="E1" s="43"/>
+      <c r="F1" s="43"/>
+      <c r="G1" s="43"/>
+      <c r="H1" s="43"/>
+      <c r="I1" s="43"/>
       <c r="N1" s="2" t="s">
         <v>1</v>
       </c>
@@ -1366,15 +1378,15 @@
       </c>
     </row>
     <row r="2" spans="1:15" ht="17.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C2" s="43" t="s">
+      <c r="C2" s="44" t="s">
         <v>3</v>
       </c>
-      <c r="D2" s="43"/>
-      <c r="E2" s="43"/>
-      <c r="F2" s="43"/>
-      <c r="G2" s="43"/>
-      <c r="H2" s="43"/>
-      <c r="I2" s="43"/>
+      <c r="D2" s="44"/>
+      <c r="E2" s="44"/>
+      <c r="F2" s="44"/>
+      <c r="G2" s="44"/>
+      <c r="H2" s="44"/>
+      <c r="I2" s="44"/>
       <c r="J2" s="3"/>
       <c r="L2" s="3"/>
       <c r="N2" s="2" t="s">
@@ -1385,50 +1397,50 @@
       </c>
     </row>
     <row r="3" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C3" s="44" t="s">
+      <c r="C3" s="45" t="s">
         <v>6</v>
       </c>
-      <c r="D3" s="44"/>
-      <c r="E3" s="44"/>
-      <c r="F3" s="44"/>
-      <c r="G3" s="44"/>
-      <c r="H3" s="44"/>
-      <c r="I3" s="44"/>
+      <c r="D3" s="45"/>
+      <c r="E3" s="45"/>
+      <c r="F3" s="45"/>
+      <c r="G3" s="45"/>
+      <c r="H3" s="45"/>
+      <c r="I3" s="45"/>
       <c r="J3" s="4"/>
       <c r="L3" s="4"/>
     </row>
     <row r="4" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="C4" s="45" t="s">
+      <c r="C4" s="46" t="s">
         <v>7</v>
       </c>
-      <c r="D4" s="45"/>
-      <c r="E4" s="45"/>
-      <c r="F4" s="45"/>
-      <c r="G4" s="45"/>
-      <c r="H4" s="45"/>
-      <c r="I4" s="45"/>
+      <c r="D4" s="46"/>
+      <c r="E4" s="46"/>
+      <c r="F4" s="46"/>
+      <c r="G4" s="46"/>
+      <c r="H4" s="46"/>
+      <c r="I4" s="46"/>
     </row>
     <row r="5" spans="1:15" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C5" s="46" t="s">
+      <c r="C5" s="47" t="s">
         <v>8</v>
       </c>
-      <c r="D5" s="46"/>
-      <c r="E5" s="46"/>
-      <c r="F5" s="46"/>
-      <c r="G5" s="46"/>
-      <c r="H5" s="46"/>
-      <c r="I5" s="46"/>
+      <c r="D5" s="47"/>
+      <c r="E5" s="47"/>
+      <c r="F5" s="47"/>
+      <c r="G5" s="47"/>
+      <c r="H5" s="47"/>
+      <c r="I5" s="47"/>
     </row>
     <row r="6" spans="1:15" ht="12" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C6" s="46" t="s">
+      <c r="C6" s="47" t="s">
         <v>9</v>
       </c>
-      <c r="D6" s="46"/>
-      <c r="E6" s="46"/>
-      <c r="F6" s="46"/>
-      <c r="G6" s="46"/>
-      <c r="H6" s="46"/>
-      <c r="I6" s="46"/>
+      <c r="D6" s="47"/>
+      <c r="E6" s="47"/>
+      <c r="F6" s="47"/>
+      <c r="G6" s="47"/>
+      <c r="H6" s="47"/>
+      <c r="I6" s="47"/>
       <c r="J6" s="5"/>
       <c r="L6" s="5"/>
     </row>
@@ -1484,32 +1496,32 @@
     </row>
     <row r="12" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A12" s="11"/>
-      <c r="B12" s="53" t="s">
+      <c r="B12" s="54" t="s">
         <v>12</v>
       </c>
-      <c r="C12" s="47" t="s">
+      <c r="C12" s="48" t="s">
         <v>13</v>
       </c>
-      <c r="D12" s="48"/>
+      <c r="D12" s="49"/>
       <c r="E12" s="12"/>
-      <c r="F12" s="47" t="s">
+      <c r="F12" s="48" t="s">
         <v>14</v>
       </c>
-      <c r="G12" s="48"/>
-      <c r="H12" s="49"/>
+      <c r="G12" s="49"/>
+      <c r="H12" s="50"/>
       <c r="I12" s="13" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="13" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A13" s="11"/>
-      <c r="B13" s="54"/>
-      <c r="C13" s="50"/>
-      <c r="D13" s="51"/>
+      <c r="B13" s="55"/>
+      <c r="C13" s="51"/>
+      <c r="D13" s="52"/>
       <c r="E13" s="11"/>
-      <c r="F13" s="50"/>
-      <c r="G13" s="51"/>
-      <c r="H13" s="52"/>
+      <c r="F13" s="51"/>
+      <c r="G13" s="52"/>
+      <c r="H13" s="53"/>
       <c r="I13" s="14" t="s">
         <v>16</v>
       </c>
@@ -1519,16 +1531,16 @@
       <c r="B14" s="16">
         <v>1</v>
       </c>
-      <c r="C14" s="55" t="s">
+      <c r="C14" s="56" t="s">
         <v>17</v>
       </c>
-      <c r="D14" s="56"/>
-      <c r="E14" s="57"/>
-      <c r="F14" s="58" t="s">
+      <c r="D14" s="57"/>
+      <c r="E14" s="58"/>
+      <c r="F14" s="59" t="s">
         <v>18</v>
       </c>
-      <c r="G14" s="58"/>
-      <c r="H14" s="58"/>
+      <c r="G14" s="59"/>
+      <c r="H14" s="59"/>
       <c r="I14" s="17" t="s">
         <v>19</v>
       </c>
@@ -1538,16 +1550,16 @@
       <c r="B15" s="18">
         <v>2</v>
       </c>
-      <c r="C15" s="59" t="s">
+      <c r="C15" s="60" t="s">
         <v>20</v>
       </c>
-      <c r="D15" s="60"/>
-      <c r="E15" s="61"/>
-      <c r="F15" s="62" t="s">
+      <c r="D15" s="61"/>
+      <c r="E15" s="62"/>
+      <c r="F15" s="63" t="s">
         <v>21</v>
       </c>
-      <c r="G15" s="62"/>
-      <c r="H15" s="62"/>
+      <c r="G15" s="63"/>
+      <c r="H15" s="63"/>
       <c r="I15" s="20" t="s">
         <v>19</v>
       </c>
@@ -1557,16 +1569,16 @@
       <c r="B16" s="18">
         <v>3</v>
       </c>
-      <c r="C16" s="59" t="s">
+      <c r="C16" s="60" t="s">
         <v>22</v>
       </c>
-      <c r="D16" s="60"/>
-      <c r="E16" s="61"/>
-      <c r="F16" s="62" t="s">
+      <c r="D16" s="61"/>
+      <c r="E16" s="62"/>
+      <c r="F16" s="63" t="s">
         <v>23</v>
       </c>
-      <c r="G16" s="62"/>
-      <c r="H16" s="62"/>
+      <c r="G16" s="63"/>
+      <c r="H16" s="63"/>
       <c r="I16" s="20" t="s">
         <v>19</v>
       </c>
@@ -1574,58 +1586,58 @@
     <row r="17" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A17" s="11"/>
       <c r="B17" s="21"/>
-      <c r="C17" s="59"/>
-      <c r="D17" s="60"/>
-      <c r="E17" s="61"/>
-      <c r="F17" s="62"/>
-      <c r="G17" s="62"/>
-      <c r="H17" s="62"/>
+      <c r="C17" s="60"/>
+      <c r="D17" s="61"/>
+      <c r="E17" s="62"/>
+      <c r="F17" s="63"/>
+      <c r="G17" s="63"/>
+      <c r="H17" s="63"/>
       <c r="I17" s="22"/>
       <c r="J17" s="23"/>
     </row>
     <row r="18" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A18" s="11"/>
       <c r="B18" s="21"/>
-      <c r="C18" s="59"/>
-      <c r="D18" s="60"/>
-      <c r="E18" s="61"/>
-      <c r="F18" s="62"/>
-      <c r="G18" s="62"/>
-      <c r="H18" s="62"/>
+      <c r="C18" s="60"/>
+      <c r="D18" s="61"/>
+      <c r="E18" s="62"/>
+      <c r="F18" s="63"/>
+      <c r="G18" s="63"/>
+      <c r="H18" s="63"/>
       <c r="I18" s="22"/>
       <c r="J18" s="23"/>
     </row>
     <row r="19" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A19" s="11"/>
       <c r="B19" s="21"/>
-      <c r="C19" s="59"/>
-      <c r="D19" s="60"/>
-      <c r="E19" s="61"/>
-      <c r="F19" s="62"/>
-      <c r="G19" s="62"/>
-      <c r="H19" s="62"/>
+      <c r="C19" s="60"/>
+      <c r="D19" s="61"/>
+      <c r="E19" s="62"/>
+      <c r="F19" s="63"/>
+      <c r="G19" s="63"/>
+      <c r="H19" s="63"/>
       <c r="I19" s="20"/>
     </row>
     <row r="20" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A20" s="11"/>
       <c r="B20" s="21"/>
-      <c r="C20" s="59"/>
-      <c r="D20" s="60"/>
-      <c r="E20" s="61"/>
-      <c r="F20" s="62"/>
-      <c r="G20" s="62"/>
-      <c r="H20" s="62"/>
+      <c r="C20" s="60"/>
+      <c r="D20" s="61"/>
+      <c r="E20" s="62"/>
+      <c r="F20" s="63"/>
+      <c r="G20" s="63"/>
+      <c r="H20" s="63"/>
       <c r="I20" s="20"/>
     </row>
     <row r="21" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="15"/>
       <c r="B21" s="24"/>
-      <c r="C21" s="63"/>
-      <c r="D21" s="64"/>
-      <c r="E21" s="65"/>
-      <c r="F21" s="66"/>
-      <c r="G21" s="67"/>
-      <c r="H21" s="68"/>
+      <c r="C21" s="64"/>
+      <c r="D21" s="65"/>
+      <c r="E21" s="66"/>
+      <c r="F21" s="67"/>
+      <c r="G21" s="68"/>
+      <c r="H21" s="69"/>
       <c r="I21" s="25"/>
     </row>
     <row r="22" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -1690,7 +1702,7 @@
       <c r="G26" s="7"/>
       <c r="H26" s="7"/>
     </row>
-    <row r="27" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A27" s="7"/>
       <c r="B27" s="31" t="s">
         <v>30</v>
@@ -1704,7 +1716,7 @@
       </c>
       <c r="H27" s="7"/>
     </row>
-    <row r="28" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A28" s="7"/>
       <c r="B28" s="31" t="s">
         <v>32</v>
@@ -1713,19 +1725,19 @@
       <c r="D28" s="7" t="s">
         <v>26</v>
       </c>
-      <c r="E28" s="69">
+      <c r="E28" s="70">
         <v>46128</v>
       </c>
-      <c r="F28" s="69"/>
+      <c r="F28" s="70"/>
       <c r="G28" s="31" t="s">
         <v>33</v>
       </c>
-      <c r="H28" s="69">
+      <c r="H28" s="70">
         <v>46128</v>
       </c>
-      <c r="I28" s="69"/>
-    </row>
-    <row r="29" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="I28" s="70"/>
+    </row>
+    <row r="29" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A29" s="7"/>
       <c r="B29" s="31" t="s">
         <v>34</v>
@@ -1734,12 +1746,12 @@
       <c r="D29" s="7" t="s">
         <v>26</v>
       </c>
-      <c r="E29" s="72"/>
-      <c r="F29" s="72"/>
+      <c r="E29" s="71"/>
+      <c r="F29" s="71"/>
       <c r="G29" s="7"/>
       <c r="H29" s="7"/>
     </row>
-    <row r="30" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A30" s="7"/>
       <c r="B30" s="7"/>
       <c r="C30" s="32"/>
@@ -1749,7 +1761,7 @@
       <c r="G30" s="7"/>
       <c r="H30" s="7"/>
     </row>
-    <row r="31" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A31" s="7"/>
       <c r="B31" s="7"/>
       <c r="C31" s="7"/>
@@ -1761,7 +1773,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="32" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A32" s="7"/>
       <c r="B32" s="7" t="s">
         <v>36</v>
@@ -1775,7 +1787,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="33" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A33" s="7"/>
       <c r="B33" s="7" t="s">
         <v>38</v>
@@ -1789,7 +1801,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="34" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A34" s="7"/>
       <c r="B34" s="7"/>
       <c r="C34" s="7"/>
@@ -1864,7 +1876,7 @@
     </row>
     <row r="40" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A40" s="32" t="s">
-        <v>61</v>
+        <v>44</v>
       </c>
       <c r="B40" s="7"/>
       <c r="C40" s="7"/>
@@ -1876,14 +1888,14 @@
     </row>
     <row r="41" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A41" s="32" t="s">
-        <v>62</v>
+        <v>45</v>
       </c>
       <c r="B41" s="7"/>
       <c r="C41" s="7"/>
       <c r="D41" s="7"/>
       <c r="E41" s="7"/>
       <c r="F41" s="36" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="G41" s="7"/>
       <c r="H41" s="7"/>
@@ -1900,20 +1912,20 @@
     </row>
     <row r="43" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A43" s="11" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="B43" s="7" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="C43" s="7"/>
-      <c r="E43" s="84" t="s">
-        <v>60</v>
+      <c r="E43" s="37" t="s">
+        <v>49</v>
       </c>
       <c r="F43" s="7" t="s">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="G43" s="7"/>
-      <c r="H43" s="37"/>
+      <c r="H43" s="38"/>
     </row>
     <row r="44" spans="1:10" ht="22" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A44" s="11"/>
@@ -1926,19 +1938,19 @@
     </row>
     <row r="45" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A45" s="11" t="s">
-        <v>48</v>
+        <v>51</v>
       </c>
       <c r="B45" s="7" t="s">
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="C45" s="7"/>
-      <c r="E45" s="84" t="s">
-        <v>59</v>
-      </c>
-      <c r="F45" s="83">
+      <c r="E45" s="37" t="s">
+        <v>53</v>
+      </c>
+      <c r="F45" s="72">
         <v>1590000</v>
       </c>
-      <c r="G45" s="83"/>
+      <c r="G45" s="72"/>
       <c r="H45" s="7"/>
     </row>
     <row r="46" spans="1:10" ht="22" customHeight="1" x14ac:dyDescent="0.35">
@@ -1953,18 +1965,18 @@
     </row>
     <row r="47" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A47" s="11" t="s">
-        <v>50</v>
+        <v>54</v>
       </c>
       <c r="B47" s="7" t="s">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="C47" s="32"/>
       <c r="D47" s="32"/>
-      <c r="E47" s="84" t="s">
-        <v>59</v>
+      <c r="E47" s="37" t="s">
+        <v>53</v>
       </c>
       <c r="F47" s="7" t="s">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="G47" s="7"/>
       <c r="H47" s="7"/>
@@ -1981,18 +1993,18 @@
     </row>
     <row r="49" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A49" s="11" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="B49" s="7" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="C49" s="7"/>
       <c r="D49" s="7"/>
-      <c r="E49" s="84" t="s">
-        <v>59</v>
+      <c r="E49" s="37" t="s">
+        <v>53</v>
       </c>
       <c r="F49" s="7" t="s">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="G49" s="7"/>
       <c r="H49" s="7"/>
@@ -2020,11 +2032,11 @@
     <row r="52" spans="1:9" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A52" s="7"/>
       <c r="B52" s="73" t="s">
-        <v>54</v>
+        <v>58</v>
       </c>
       <c r="C52" s="74"/>
       <c r="D52" s="77" t="s">
-        <v>55</v>
+        <v>59</v>
       </c>
       <c r="E52" s="78"/>
       <c r="F52" s="79"/>
@@ -2044,36 +2056,36 @@
     <row r="54" spans="1:9" ht="28.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A54" s="7"/>
       <c r="B54" s="19" t="s">
-        <v>56</v>
-      </c>
-      <c r="C54" s="38"/>
-      <c r="D54" s="39"/>
-      <c r="E54" s="70"/>
-      <c r="F54" s="71"/>
+        <v>60</v>
+      </c>
+      <c r="C54" s="39"/>
+      <c r="D54" s="40"/>
+      <c r="E54" s="83"/>
+      <c r="F54" s="84"/>
       <c r="G54" s="7"/>
       <c r="H54" s="7"/>
     </row>
     <row r="55" spans="1:9" ht="28.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A55" s="7"/>
       <c r="B55" s="19" t="s">
-        <v>57</v>
-      </c>
-      <c r="C55" s="38"/>
-      <c r="D55" s="40"/>
-      <c r="E55" s="70"/>
-      <c r="F55" s="71"/>
+        <v>61</v>
+      </c>
+      <c r="C55" s="39"/>
+      <c r="D55" s="41"/>
+      <c r="E55" s="83"/>
+      <c r="F55" s="84"/>
       <c r="G55" s="7"/>
       <c r="H55" s="7"/>
     </row>
     <row r="56" spans="1:9" ht="28.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A56" s="7"/>
       <c r="B56" s="19" t="s">
-        <v>58</v>
-      </c>
-      <c r="C56" s="38"/>
-      <c r="D56" s="40"/>
-      <c r="E56" s="70"/>
-      <c r="F56" s="71"/>
+        <v>62</v>
+      </c>
+      <c r="C56" s="39"/>
+      <c r="D56" s="41"/>
+      <c r="E56" s="83"/>
+      <c r="F56" s="84"/>
       <c r="G56" s="7"/>
       <c r="H56" s="7"/>
     </row>
@@ -2088,14 +2100,14 @@
       <c r="H57" s="7"/>
     </row>
     <row r="58" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A58" s="41"/>
-      <c r="B58" s="41"/>
-      <c r="C58" s="41"/>
-      <c r="D58" s="41"/>
-      <c r="E58" s="41"/>
-      <c r="F58" s="41"/>
-      <c r="G58" s="41"/>
-      <c r="H58" s="41"/>
+      <c r="A58" s="42"/>
+      <c r="B58" s="42"/>
+      <c r="C58" s="42"/>
+      <c r="D58" s="42"/>
+      <c r="E58" s="42"/>
+      <c r="F58" s="42"/>
+      <c r="G58" s="42"/>
+      <c r="H58" s="42"/>
       <c r="I58" s="6"/>
     </row>
     <row r="59" spans="1:9" x14ac:dyDescent="0.35">
@@ -2284,13 +2296,13 @@
     </row>
   </sheetData>
   <mergeCells count="35">
+    <mergeCell ref="E55:F55"/>
     <mergeCell ref="E56:F56"/>
     <mergeCell ref="E29:F29"/>
+    <mergeCell ref="F45:G45"/>
     <mergeCell ref="B52:C53"/>
     <mergeCell ref="D52:F53"/>
     <mergeCell ref="E54:F54"/>
-    <mergeCell ref="E55:F55"/>
-    <mergeCell ref="F45:G45"/>
     <mergeCell ref="C20:E20"/>
     <mergeCell ref="F20:H20"/>
     <mergeCell ref="C21:E21"/>

</xml_diff>